<commit_message>
Update published master datasets (2026-03-03)
</commit_message>
<xml_diff>
--- a/archive/InnovateUK_Funding_Opportunities_WeeklyBreakdown_2026-03-03.xlsx
+++ b/archive/InnovateUK_Funding_Opportunities_WeeklyBreakdown_2026-03-03.xlsx
@@ -482,13 +482,13 @@
         <v>46078</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -8010,7 +8010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8801,26 +8801,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 7</t>
+          <t>ARIA: Enduring Atmospheric Platforms - full proposals</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2404/overview/99693fa4-0f17-4de8-b812-34f2be37a4d0</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/aria-enduring-atmospheric-platforms-full-proposals/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-02-26 10:40</t>
+          <t>2026-03-03 10:27</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46079.44444444445</v>
+        <v>46084.43541666667</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -8829,25 +8829,137 @@
       <c r="H14" t="b">
         <v>0</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>46082</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Wednesday 8 April 2026 11:00am</t>
+          <t>02/04/2026                              12:00</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>46120.45833333334</v>
+        <v>46114.5</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£500</t>
         </is>
       </c>
       <c r="N14" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="O14" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ADOPT Facilitator Support Grant: Round 7</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2404/overview/99693fa4-0f17-4de8-b812-34f2be37a4d0</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:40</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>46079.44444444445</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Wednesday 8 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>46120.45833333334</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>£2,500</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>46078</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SNPN 5G Assured Integration (CR&amp;D)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2400/overview/cbbc48e2-d78e-42cd-b570-330f702ba82f</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-03-03 10:34</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>46084.44027777778</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Wednesday 1 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>46113.45833333334</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>£4.0 million</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="O16" s="1" t="n">
         <v>46078</v>
       </c>
     </row>

</xml_diff>